<commit_message>
🔒 [FULL] Daily chip data 2026-09-02 03:05
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -1239,12 +1239,12 @@
     <comment ref="D17" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「陳族元」獨佔比 63.6%
-  • 領頭金額 79,367 萬
-  • 合計淨買 124,822 萬
+領頭大戶「陳族元」獨佔比 63.4%
+  • 領頭金額 78,702 萬
+  • 合計淨買 124,157 萬
   • 大戶數 10 位 (名義共識)
 判讀: 名義 10 位大戶共識,
-實質 1 人下注佔 64%,
+實質 1 人下注佔 63%,
 剩餘 9 位為陪襯小單,
 真共識訊號被稀釋.</t>
       </text>
@@ -1265,9 +1265,9 @@
     <comment ref="D20" authorId="0" shapeId="0">
       <text>
         <t>⚠️ 假共識警示
-領頭大戶「張濬安(航海王)」獨佔比 54.3%
+領頭大戶「張濬安(航海王)」獨佔比 53.6%
   • 領頭金額 24,904 萬
-  • 合計淨買 45,905 萬
+  • 合計淨買 46,428 萬
   • 大戶數 11 位 (名義共識)
 判讀: 名義 11 位大戶共識,
 實質 1 人下注佔 54%,
@@ -1795,33 +1795,33 @@
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
+          <t>張濬安</t>
+        </is>
+      </c>
+      <c r="H16" s="17" t="n">
+        <v>21508</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>陳律師</t>
+        </is>
+      </c>
+      <c r="J16" s="18" t="n">
+        <v>21175</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
           <t>陳族元</t>
         </is>
       </c>
-      <c r="H16" s="17" t="n">
-        <v>26403</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>張濬安</t>
-        </is>
-      </c>
-      <c r="J16" s="18" t="n">
-        <v>21508</v>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>陳律師</t>
-        </is>
-      </c>
       <c r="L16" s="18" t="n">
-        <v>21175</v>
+        <v>19716</v>
       </c>
       <c r="M16" s="19" t="n">
         <v>9</v>
       </c>
       <c r="N16" s="17" t="n">
-        <v>159590</v>
+        <v>152902</v>
       </c>
     </row>
     <row r="17">
@@ -1850,7 +1850,7 @@
         </is>
       </c>
       <c r="H17" s="17" t="n">
-        <v>79368</v>
+        <v>78703</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1872,7 +1872,7 @@
         <v>7</v>
       </c>
       <c r="N17" s="17" t="n">
-        <v>124823</v>
+        <v>124158</v>
       </c>
     </row>
     <row r="18">
@@ -1901,7 +1901,7 @@
         </is>
       </c>
       <c r="H18" s="17" t="n">
-        <v>13145</v>
+        <v>13887</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
         <v>10</v>
       </c>
       <c r="N18" s="17" t="n">
-        <v>77551</v>
+        <v>78294</v>
       </c>
     </row>
     <row r="19">
@@ -1995,7 +1995,7 @@
         <v>11</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
@@ -2019,13 +2019,13 @@
         </is>
       </c>
       <c r="L20" s="18" t="n">
-        <v>3481</v>
+        <v>4004</v>
       </c>
       <c r="M20" s="19" t="n">
         <v>8</v>
       </c>
       <c r="N20" s="17" t="n">
-        <v>45905</v>
+        <v>46428</v>
       </c>
     </row>
     <row r="21">
@@ -2050,33 +2050,33 @@
       </c>
       <c r="G21" s="16" t="inlineStr">
         <is>
+          <t>陳族元</t>
+        </is>
+      </c>
+      <c r="H21" s="17" t="n">
+        <v>7366</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
           <t>強森</t>
         </is>
       </c>
-      <c r="H21" s="17" t="n">
+      <c r="J21" s="18" t="n">
         <v>6655</v>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>張濬安</t>
         </is>
       </c>
-      <c r="J21" s="18" t="n">
+      <c r="L21" s="18" t="n">
         <v>6323</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>陳族元</t>
-        </is>
-      </c>
-      <c r="L21" s="18" t="n">
-        <v>6188</v>
       </c>
       <c r="M21" s="19" t="n">
         <v>9</v>
       </c>
       <c r="N21" s="17" t="n">
-        <v>32855</v>
+        <v>34034</v>
       </c>
     </row>
     <row r="22">
@@ -2121,13 +2121,13 @@
         </is>
       </c>
       <c r="L22" s="18" t="n">
-        <v>4908</v>
+        <v>4993</v>
       </c>
       <c r="M22" s="19" t="n">
         <v>10</v>
       </c>
       <c r="N22" s="17" t="n">
-        <v>32227</v>
+        <v>32312</v>
       </c>
     </row>
     <row r="23">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H24" s="17" t="n">
-        <v>8801</v>
+        <v>9943</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -2229,7 +2229,7 @@
         <v>7</v>
       </c>
       <c r="N24" s="17" t="n">
-        <v>27677</v>
+        <v>28819</v>
       </c>
     </row>
     <row r="25">
@@ -2247,10 +2247,10 @@
         </is>
       </c>
       <c r="E25" s="14" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F25" s="15" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G25" s="16" t="inlineStr">
         <is>
@@ -2277,10 +2277,10 @@
         <v>1491</v>
       </c>
       <c r="M25" s="19" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N25" s="17" t="n">
-        <v>21402</v>
+        <v>20948</v>
       </c>
     </row>
     <row r="26">
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="J26" s="18" t="n">
-        <v>3291</v>
+        <v>3239</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -2331,7 +2331,7 @@
         <v>7</v>
       </c>
       <c r="N26" s="17" t="n">
-        <v>15758</v>
+        <v>15707</v>
       </c>
     </row>
     <row r="27">
@@ -2360,7 +2360,7 @@
         </is>
       </c>
       <c r="H27" s="17" t="n">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2382,7 +2382,7 @@
         <v>7</v>
       </c>
       <c r="N27" s="17" t="n">
-        <v>2600</v>
+        <v>2601</v>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
@@ -2407,7 +2407,7 @@
         </is>
       </c>
       <c r="G30" s="211" t="n">
-        <v>-18.87241</v>
+        <v>-23.14886</v>
       </c>
     </row>
     <row r="31" ht="28" customHeight="1">
@@ -2416,7 +2416,7 @@
           <t>Q3 強共識股</t>
         </is>
       </c>
-      <c r="C31" s="240" t="n">
+      <c r="C31" s="212" t="n">
         <v>12</v>
       </c>
       <c r="F31" s="22" t="inlineStr">
@@ -2424,8 +2424,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G31" s="241" t="n">
-        <v>0.2094574796909283</v>
+      <c r="G31" s="213" t="n">
+        <v>0.2097539260421956</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -2536,11 +2536,11 @@
         </is>
       </c>
       <c r="D38" s="33" t="n">
-        <v>1489239</v>
+        <v>1485604</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>21.8%</t>
+          <t>21.7%</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2552,7 +2552,7 @@
         </is>
       </c>
       <c r="H38" s="33" t="n">
-        <v>234608</v>
+        <v>234593</v>
       </c>
       <c r="I38" s="215" t="n">
         <v>0.0271</v>
@@ -3016,11 +3016,11 @@
         <v>23</v>
       </c>
       <c r="E60" t="n">
-        <v>1130409</v>
+        <v>1127222</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>陳族元 連續 23 天加碼 3008 (累計 1,130,409 萬)</t>
+          <t>陳族元 連續 23 天加碼 3008 (累計 1,127,222 萬)</t>
         </is>
       </c>
     </row>
@@ -3237,7 +3237,7 @@
         </is>
       </c>
       <c r="C70" s="33" t="n">
-        <v>1447590</v>
+        <v>1443898</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3245,7 +3245,7 @@
         </is>
       </c>
       <c r="E70" s="33" t="n">
-        <v>124513</v>
+        <v>123706</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -3253,7 +3253,7 @@
         </is>
       </c>
       <c r="G70" s="33" t="n">
-        <v>108644</v>
+        <v>107986</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
@@ -3264,7 +3264,7 @@
         <v>94068</v>
       </c>
       <c r="J70" s="216" t="n">
-        <v>0.2260477669617202</v>
+        <v>0.2256120673385749</v>
       </c>
     </row>
     <row r="71">
@@ -4813,7 +4813,7 @@
     <row r="36" ht="22" customHeight="1">
       <c r="C36" s="73" t="inlineStr">
         <is>
-          <t>-19 億 淨買</t>
+          <t>-23 億 淨買</t>
         </is>
       </c>
     </row>
@@ -14506,27 +14506,27 @@
         </is>
       </c>
       <c r="E190" s="136" t="n">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="F190" s="136" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G190" s="136" t="n">
-        <v>29518</v>
+        <v>28712</v>
       </c>
       <c r="H190" s="136" t="n">
-        <v>9516</v>
+        <v>9406</v>
       </c>
       <c r="I190" s="136" t="n">
-        <v>20002</v>
+        <v>19306</v>
       </c>
       <c r="J190" s="137" t="n">
-        <v>971</v>
+        <v>969.99</v>
       </c>
       <c r="K190" s="137" t="n">
-        <v>971</v>
-      </c>
-      <c r="L190" s="236">
+        <v>969.74</v>
+      </c>
+      <c r="L190" s="235">
         <f>F190*(K190-J190)</f>
         <v/>
       </c>
@@ -14541,25 +14541,25 @@
         </is>
       </c>
       <c r="E191" s="136" t="n">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="F191" s="136" t="n">
         <v>3</v>
       </c>
       <c r="G191" s="136" t="n">
-        <v>20580</v>
+        <v>19923</v>
       </c>
       <c r="H191" s="136" t="n">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="I191" s="136" t="n">
-        <v>20212</v>
+        <v>19547</v>
       </c>
       <c r="J191" s="137" t="n">
-        <v>1225</v>
+        <v>1222.26</v>
       </c>
       <c r="K191" s="137" t="n">
-        <v>1225</v>
+        <v>1251.67</v>
       </c>
       <c r="L191" s="236">
         <f>F191*(K191-J191)</f>
@@ -14572,29 +14572,29 @@
       <c r="C192" s="138" t="n"/>
       <c r="D192" s="135" t="inlineStr">
         <is>
-          <t>南亞科(2408)</t>
+          <t>雙鴻(3324)</t>
         </is>
       </c>
       <c r="E192" s="136" t="n">
-        <v>214</v>
+        <v>60</v>
       </c>
       <c r="F192" s="136" t="n">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="G192" s="136" t="n">
-        <v>11069</v>
+        <v>8188</v>
       </c>
       <c r="H192" s="136" t="n">
-        <v>2719</v>
+        <v>1802</v>
       </c>
       <c r="I192" s="136" t="n">
-        <v>8350</v>
+        <v>6386</v>
       </c>
       <c r="J192" s="137" t="n">
-        <v>517.22</v>
+        <v>1364.62</v>
       </c>
       <c r="K192" s="137" t="n">
-        <v>522.9400000000001</v>
+        <v>1386.15</v>
       </c>
       <c r="L192" s="236">
         <f>F192*(K192-J192)</f>
@@ -14607,31 +14607,31 @@
       <c r="C193" s="138" t="n"/>
       <c r="D193" s="135" t="inlineStr">
         <is>
-          <t>雙鴻(3324)</t>
+          <t>智邦(2345)</t>
         </is>
       </c>
       <c r="E193" s="136" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="F193" s="136" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G193" s="136" t="n">
-        <v>8250</v>
+        <v>4268</v>
       </c>
       <c r="H193" s="136" t="n">
-        <v>1925</v>
+        <v>25</v>
       </c>
       <c r="I193" s="136" t="n">
-        <v>6325</v>
+        <v>4243</v>
       </c>
       <c r="J193" s="137" t="n">
-        <v>1375</v>
+        <v>2246.47</v>
       </c>
       <c r="K193" s="137" t="n">
-        <v>1375</v>
-      </c>
-      <c r="L193" s="236">
+        <v>252</v>
+      </c>
+      <c r="L193" s="235">
         <f>F193*(K193-J193)</f>
         <v/>
       </c>
@@ -14642,31 +14642,31 @@
       <c r="C194" s="138" t="n"/>
       <c r="D194" s="135" t="inlineStr">
         <is>
-          <t>金居(8358)</t>
+          <t>南亞(1303)</t>
         </is>
       </c>
       <c r="E194" s="136" t="n">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="F194" s="136" t="n">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="G194" s="136" t="n">
-        <v>4058</v>
+        <v>3867</v>
       </c>
       <c r="H194" s="136" t="n">
-        <v>3595</v>
+        <v>1838</v>
       </c>
       <c r="I194" s="136" t="n">
-        <v>463</v>
+        <v>2029</v>
       </c>
       <c r="J194" s="137" t="n">
-        <v>527.04</v>
+        <v>444.47</v>
       </c>
       <c r="K194" s="137" t="n">
-        <v>528.6900000000001</v>
-      </c>
-      <c r="L194" s="236">
+        <v>353.52</v>
+      </c>
+      <c r="L194" s="235">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -14677,29 +14677,29 @@
       <c r="C195" s="138" t="n"/>
       <c r="D195" s="135" t="inlineStr">
         <is>
-          <t>台虹(8039)</t>
+          <t>緯穎(6669)</t>
         </is>
       </c>
       <c r="E195" s="136" t="n">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="F195" s="136" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="G195" s="136" t="n">
-        <v>3430</v>
+        <v>3825</v>
       </c>
       <c r="H195" s="136" t="n">
-        <v>1959</v>
+        <v>3271</v>
       </c>
       <c r="I195" s="136" t="n">
-        <v>1471</v>
+        <v>554</v>
       </c>
       <c r="J195" s="137" t="n">
-        <v>623.58</v>
+        <v>7649.2</v>
       </c>
       <c r="K195" s="137" t="n">
-        <v>1088.33</v>
+        <v>8177.75</v>
       </c>
       <c r="L195" s="236">
         <f>F195*(K195-J195)</f>
@@ -14712,29 +14712,29 @@
       <c r="C196" s="138" t="n"/>
       <c r="D196" s="135" t="inlineStr">
         <is>
-          <t>旺矽(6223)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="E196" s="136" t="n">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="F196" s="136" t="n">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="G196" s="136" t="n">
-        <v>3243</v>
+        <v>2893</v>
       </c>
       <c r="H196" s="136" t="n">
-        <v>635</v>
+        <v>1231</v>
       </c>
       <c r="I196" s="136" t="n">
-        <v>2608</v>
+        <v>1662</v>
       </c>
       <c r="J196" s="137" t="n">
-        <v>5404.33</v>
+        <v>137.1</v>
       </c>
       <c r="K196" s="137" t="n">
-        <v>6354</v>
+        <v>236.73</v>
       </c>
       <c r="L196" s="236">
         <f>F196*(K196-J196)</f>
@@ -14747,29 +14747,29 @@
       <c r="C197" s="138" t="n"/>
       <c r="D197" s="135" t="inlineStr">
         <is>
-          <t>大立光(3008)</t>
+          <t>大量(3167)</t>
         </is>
       </c>
       <c r="E197" s="136" t="n">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="F197" s="136" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="G197" s="136" t="n">
-        <v>3187</v>
+        <v>2657</v>
       </c>
       <c r="H197" s="136" t="n">
-        <v>208</v>
+        <v>1678</v>
       </c>
       <c r="I197" s="136" t="n">
-        <v>2979</v>
+        <v>979</v>
       </c>
       <c r="J197" s="137" t="n">
-        <v>7966.75</v>
+        <v>805.09</v>
       </c>
       <c r="K197" s="137" t="n">
-        <v>2081</v>
+        <v>798.86</v>
       </c>
       <c r="L197" s="235">
         <f>F197*(K197-J197)</f>
@@ -14786,27 +14786,27 @@
         </is>
       </c>
       <c r="E198" s="136" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F198" s="136" t="n">
         <v>1</v>
       </c>
       <c r="G198" s="136" t="n">
-        <v>2475</v>
+        <v>2423</v>
       </c>
       <c r="H198" s="136" t="n">
         <v>28</v>
       </c>
       <c r="I198" s="136" t="n">
-        <v>2447</v>
+        <v>2395</v>
       </c>
       <c r="J198" s="137" t="n">
-        <v>278.04</v>
+        <v>278.51</v>
       </c>
       <c r="K198" s="137" t="n">
-        <v>282</v>
-      </c>
-      <c r="L198" s="236">
+        <v>278</v>
+      </c>
+      <c r="L198" s="235">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>
@@ -14817,29 +14817,29 @@
       <c r="C199" s="138" t="n"/>
       <c r="D199" s="135" t="inlineStr">
         <is>
-          <t>聯亞(3081)</t>
+          <t>金居(8358)</t>
         </is>
       </c>
       <c r="E199" s="136" t="n">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="F199" s="136" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G199" s="136" t="n">
-        <v>2470</v>
+        <v>2096</v>
       </c>
       <c r="H199" s="136" t="n">
-        <v>393</v>
+        <v>490</v>
       </c>
       <c r="I199" s="136" t="n">
-        <v>2077</v>
+        <v>1606</v>
       </c>
       <c r="J199" s="137" t="n">
-        <v>3528.29</v>
+        <v>523.9</v>
       </c>
       <c r="K199" s="137" t="n">
-        <v>3926</v>
+        <v>544.89</v>
       </c>
       <c r="L199" s="236">
         <f>F199*(K199-J199)</f>
@@ -23016,33 +23016,33 @@
       <c r="A414" s="185" t="n"/>
       <c r="B414" s="185" t="n"/>
       <c r="C414" s="185" t="n"/>
-      <c r="D414" s="186" t="inlineStr">
+      <c r="D414" s="182" t="inlineStr">
         <is>
           <t>和桐(1714)</t>
         </is>
       </c>
-      <c r="E414" s="187" t="n">
+      <c r="E414" s="183" t="n">
         <v>11101</v>
       </c>
-      <c r="F414" s="187" t="n">
+      <c r="F414" s="183" t="n">
         <v>3418</v>
       </c>
-      <c r="G414" s="187" t="n">
+      <c r="G414" s="183" t="n">
         <v>20592</v>
       </c>
-      <c r="H414" s="187" t="n">
+      <c r="H414" s="183" t="n">
         <v>6341</v>
       </c>
-      <c r="I414" s="187" t="n">
+      <c r="I414" s="183" t="n">
         <v>14251</v>
       </c>
-      <c r="J414" s="188" t="n">
+      <c r="J414" s="184" t="n">
         <v>18.55</v>
       </c>
-      <c r="K414" s="188" t="n">
+      <c r="K414" s="184" t="n">
         <v>18.55</v>
       </c>
-      <c r="L414" s="238">
+      <c r="L414" s="236">
         <f>F414*(K414-J414)</f>
         <v/>
       </c>
@@ -23191,33 +23191,33 @@
       <c r="A419" s="185" t="n"/>
       <c r="B419" s="185" t="n"/>
       <c r="C419" s="185" t="n"/>
-      <c r="D419" s="182" t="inlineStr">
+      <c r="D419" s="186" t="inlineStr">
         <is>
           <t>亞信(3169)</t>
         </is>
       </c>
-      <c r="E419" s="183" t="n">
+      <c r="E419" s="187" t="n">
         <v>141</v>
       </c>
-      <c r="F419" s="183" t="n">
+      <c r="F419" s="187" t="n">
         <v>0</v>
       </c>
-      <c r="G419" s="183" t="n">
+      <c r="G419" s="187" t="n">
         <v>1558</v>
       </c>
-      <c r="H419" s="183" t="n">
+      <c r="H419" s="187" t="n">
         <v>0</v>
       </c>
-      <c r="I419" s="183" t="n">
+      <c r="I419" s="187" t="n">
         <v>1558</v>
       </c>
-      <c r="J419" s="184" t="n">
+      <c r="J419" s="188" t="n">
         <v>110.5</v>
       </c>
-      <c r="K419" s="184" t="n">
+      <c r="K419" s="188" t="n">
         <v>0</v>
       </c>
-      <c r="L419" s="236">
+      <c r="L419" s="238">
         <f>F419*(K419-J419)</f>
         <v/>
       </c>
@@ -25448,7 +25448,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="207" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-09-01 18:10 | 6/17 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-09-01 19:05 | 6/17 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-09-03 02:14
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -22,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="19">
+  <numFmts count="21">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-177/5d-99)&quot;;-0&quot; 億 (昨-177/5d-99)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +63億 &quot;&quot;(昨15/5d11)&quot;"/>
@@ -42,6 +42,8 @@
     <numFmt numFmtId="180" formatCode="0&quot; 檔 +120億 &quot;&quot;(昨12/5d11)&quot;"/>
     <numFmt numFmtId="181" formatCode="0.0%&quot; 市-1611億 &quot;&quot;(昨21/5d19)&quot;"/>
     <numFmt numFmtId="182" formatCode="&quot;📅 明日預測 ↕ 中性 &quot;0.0&quot;% 信心 — P/C Ratio 主推 — 3 檔焦點&quot;"/>
+    <numFmt numFmtId="183" formatCode="0&quot; 檔 +121億 &quot;&quot;(昨12/5d11)&quot;"/>
+    <numFmt numFmtId="184" formatCode="0.0%&quot; 市-1608億 &quot;&quot;(昨21/5d19)&quot;"/>
   </numFmts>
   <fonts count="52">
     <font>
@@ -612,7 +614,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="248">
+  <cellXfs count="250">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1185,6 +1187,12 @@
     </xf>
     <xf numFmtId="171" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="51" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="183" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="184" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1870,10 +1878,10 @@
         </is>
       </c>
       <c r="E17" s="14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G17" s="16" t="inlineStr">
         <is>
@@ -1900,10 +1908,10 @@
         <v>40732</v>
       </c>
       <c r="M17" s="19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N17" s="17" t="n">
-        <v>256864</v>
+        <v>268406</v>
       </c>
     </row>
     <row r="18">
@@ -2638,23 +2646,23 @@
         <v>10</v>
       </c>
       <c r="F32" s="15" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G32" s="16" t="inlineStr">
         <is>
+          <t>陳族元</t>
+        </is>
+      </c>
+      <c r="H32" s="17" t="n">
+        <v>2382</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
           <t>強森</t>
         </is>
       </c>
-      <c r="H32" s="17" t="n">
+      <c r="J32" s="18" t="n">
         <v>1370</v>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>陳族元</t>
-        </is>
-      </c>
-      <c r="J32" s="18" t="n">
-        <v>949</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -2668,7 +2676,7 @@
         <v>7</v>
       </c>
       <c r="N32" s="17" t="n">
-        <v>5185</v>
+        <v>6618</v>
       </c>
     </row>
     <row r="33">
@@ -2737,10 +2745,10 @@
         </is>
       </c>
       <c r="E34" s="14" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F34" s="15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G34" s="16" t="inlineStr">
         <is>
@@ -2767,10 +2775,10 @@
         <v>132</v>
       </c>
       <c r="M34" s="19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N34" s="17" t="n">
-        <v>1608</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
@@ -2795,7 +2803,7 @@
         </is>
       </c>
       <c r="G37" s="242" t="n">
-        <v>-151.23464</v>
+        <v>-148.32073</v>
       </c>
     </row>
     <row r="38" ht="28" customHeight="1">
@@ -2804,7 +2812,7 @@
           <t>Q3 強共識股</t>
         </is>
       </c>
-      <c r="C38" s="243" t="n">
+      <c r="C38" s="248" t="n">
         <v>19</v>
       </c>
       <c r="F38" s="22" t="inlineStr">
@@ -2812,8 +2820,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G38" s="244" t="n">
-        <v>0.2027315599898919</v>
+      <c r="G38" s="249" t="n">
+        <v>0.2035157242394799</v>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
@@ -2896,7 +2904,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>26.8%</t>
+          <t>26.7%</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -2924,11 +2932,11 @@
         </is>
       </c>
       <c r="D45" s="33" t="n">
-        <v>929828</v>
+        <v>951729</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>21.0%</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -2940,7 +2948,7 @@
         </is>
       </c>
       <c r="H45" s="33" t="n">
-        <v>256864</v>
+        <v>268406</v>
       </c>
       <c r="I45" s="233" t="n">
         <v>-0.009300000000000001</v>
@@ -2960,7 +2968,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>12.1%</t>
+          <t>12.0%</t>
         </is>
       </c>
       <c r="F46" t="n">
@@ -2992,7 +3000,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>8.4%</t>
+          <t>8.3%</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -3024,7 +3032,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>6.7%</t>
+          <t>6.6%</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -3138,7 +3146,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>陳律師</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3148,12 +3156,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 14 檔新標的 (過去從沒買過)</t>
+          <t>陳律師 今日買進 13 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>14 檔</t>
+          <t>13 檔</t>
         </is>
       </c>
     </row>
@@ -3165,7 +3173,7 @@
       </c>
       <c r="C56" s="40" t="inlineStr">
         <is>
-          <t>陳律師</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D56" s="40" t="inlineStr">
@@ -3175,7 +3183,7 @@
       </c>
       <c r="E56" s="40" t="inlineStr">
         <is>
-          <t>陳律師 今日買進 13 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 13 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F56" s="40" t="inlineStr">
@@ -3627,7 +3635,7 @@
         </is>
       </c>
       <c r="C77" s="33" t="n">
-        <v>877076</v>
+        <v>900821</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3654,7 +3662,7 @@
         <v>76726</v>
       </c>
       <c r="J77" s="216" t="n">
-        <v>0.2905248472737998</v>
+        <v>0.28286672585709</v>
       </c>
     </row>
     <row r="78">
@@ -5046,7 +5054,7 @@
     <row r="9">
       <c r="C9" s="69" t="inlineStr">
         <is>
-          <t>② 聯發科 (2454) · 10 大戶</t>
+          <t>② 聯發科 (2454) · 11 大戶</t>
         </is>
       </c>
     </row>
@@ -5158,7 +5166,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="C29" s="73" t="inlineStr">
         <is>
-          <t>-151 億 淨買</t>
+          <t>-148 億 淨買</t>
         </is>
       </c>
     </row>
@@ -15290,29 +15298,29 @@
       </c>
       <c r="D189" s="135" t="inlineStr">
         <is>
-          <t>全新(2455)</t>
+          <t>聯發科(2454)</t>
         </is>
       </c>
       <c r="E189" s="136" t="n">
-        <v>276</v>
+        <v>50</v>
       </c>
       <c r="F189" s="136" t="n">
-        <v>245</v>
+        <v>23</v>
       </c>
       <c r="G189" s="136" t="n">
-        <v>14958</v>
+        <v>21375</v>
       </c>
       <c r="H189" s="136" t="n">
-        <v>13291</v>
+        <v>9832</v>
       </c>
       <c r="I189" s="136" t="n">
-        <v>1667</v>
+        <v>11543</v>
       </c>
       <c r="J189" s="137" t="n">
-        <v>541.97</v>
+        <v>4275</v>
       </c>
       <c r="K189" s="137" t="n">
-        <v>542.49</v>
+        <v>4275</v>
       </c>
       <c r="L189" s="236">
         <f>F189*(K189-J189)</f>
@@ -15325,29 +15333,29 @@
       <c r="C190" s="138" t="n"/>
       <c r="D190" s="135" t="inlineStr">
         <is>
-          <t>華星光(4979)</t>
+          <t>全新(2455)</t>
         </is>
       </c>
       <c r="E190" s="136" t="n">
-        <v>90</v>
+        <v>276</v>
       </c>
       <c r="F190" s="136" t="n">
-        <v>0</v>
+        <v>245</v>
       </c>
       <c r="G190" s="136" t="n">
-        <v>5539</v>
+        <v>14958</v>
       </c>
       <c r="H190" s="136" t="n">
-        <v>0</v>
+        <v>13291</v>
       </c>
       <c r="I190" s="136" t="n">
-        <v>5539</v>
+        <v>1667</v>
       </c>
       <c r="J190" s="137" t="n">
-        <v>615.4</v>
+        <v>541.97</v>
       </c>
       <c r="K190" s="137" t="n">
-        <v>0</v>
+        <v>542.49</v>
       </c>
       <c r="L190" s="236">
         <f>F190*(K190-J190)</f>
@@ -15360,29 +15368,29 @@
       <c r="C191" s="138" t="n"/>
       <c r="D191" s="135" t="inlineStr">
         <is>
-          <t>禾伸堂(3026)</t>
+          <t>華星光(4979)</t>
         </is>
       </c>
       <c r="E191" s="136" t="n">
-        <v>68</v>
+        <v>89</v>
       </c>
       <c r="F191" s="136" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="G191" s="136" t="n">
-        <v>4669</v>
+        <v>5539</v>
       </c>
       <c r="H191" s="136" t="n">
-        <v>1652</v>
+        <v>0</v>
       </c>
       <c r="I191" s="136" t="n">
-        <v>3017</v>
+        <v>5539</v>
       </c>
       <c r="J191" s="137" t="n">
-        <v>686.62</v>
+        <v>622.3099999999999</v>
       </c>
       <c r="K191" s="137" t="n">
-        <v>688.33</v>
+        <v>0</v>
       </c>
       <c r="L191" s="236">
         <f>F191*(K191-J191)</f>
@@ -15395,29 +15403,29 @@
       <c r="C192" s="138" t="n"/>
       <c r="D192" s="135" t="inlineStr">
         <is>
-          <t>台光電(2383)</t>
+          <t>禾伸堂(3026)</t>
         </is>
       </c>
       <c r="E192" s="136" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="F192" s="136" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="G192" s="136" t="n">
-        <v>4447</v>
+        <v>4669</v>
       </c>
       <c r="H192" s="136" t="n">
-        <v>0</v>
+        <v>1652</v>
       </c>
       <c r="I192" s="136" t="n">
-        <v>4447</v>
+        <v>3017</v>
       </c>
       <c r="J192" s="137" t="n">
-        <v>5559.12</v>
+        <v>686.62</v>
       </c>
       <c r="K192" s="137" t="n">
-        <v>0</v>
+        <v>688.33</v>
       </c>
       <c r="L192" s="236">
         <f>F192*(K192-J192)</f>
@@ -15430,29 +15438,29 @@
       <c r="C193" s="138" t="n"/>
       <c r="D193" s="135" t="inlineStr">
         <is>
-          <t>南亞(1303)</t>
+          <t>台光電(2383)</t>
         </is>
       </c>
       <c r="E193" s="136" t="n">
-        <v>170</v>
+        <v>8</v>
       </c>
       <c r="F193" s="136" t="n">
-        <v>143</v>
+        <v>0</v>
       </c>
       <c r="G193" s="136" t="n">
-        <v>4045</v>
+        <v>4447</v>
       </c>
       <c r="H193" s="136" t="n">
-        <v>3405</v>
+        <v>0</v>
       </c>
       <c r="I193" s="136" t="n">
-        <v>640</v>
+        <v>4447</v>
       </c>
       <c r="J193" s="137" t="n">
-        <v>237.96</v>
+        <v>5559.12</v>
       </c>
       <c r="K193" s="137" t="n">
-        <v>238.12</v>
+        <v>0</v>
       </c>
       <c r="L193" s="236">
         <f>F193*(K193-J193)</f>
@@ -15465,31 +15473,31 @@
       <c r="C194" s="138" t="n"/>
       <c r="D194" s="135" t="inlineStr">
         <is>
-          <t>台積電(2330)</t>
+          <t>南亞(1303)</t>
         </is>
       </c>
       <c r="E194" s="136" t="n">
-        <v>16</v>
+        <v>170</v>
       </c>
       <c r="F194" s="136" t="n">
-        <v>2</v>
+        <v>143</v>
       </c>
       <c r="G194" s="136" t="n">
-        <v>3933</v>
+        <v>4045</v>
       </c>
       <c r="H194" s="136" t="n">
-        <v>363</v>
+        <v>3405</v>
       </c>
       <c r="I194" s="136" t="n">
-        <v>3570</v>
+        <v>640</v>
       </c>
       <c r="J194" s="137" t="n">
-        <v>2458.12</v>
+        <v>237.96</v>
       </c>
       <c r="K194" s="137" t="n">
-        <v>1814</v>
-      </c>
-      <c r="L194" s="235">
+        <v>238.12</v>
+      </c>
+      <c r="L194" s="236">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -15500,31 +15508,31 @@
       <c r="C195" s="138" t="n"/>
       <c r="D195" s="135" t="inlineStr">
         <is>
-          <t>台燿(6274)</t>
+          <t>台積電(2330)</t>
         </is>
       </c>
       <c r="E195" s="136" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F195" s="136" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G195" s="136" t="n">
-        <v>3635</v>
+        <v>3933</v>
       </c>
       <c r="H195" s="136" t="n">
-        <v>188</v>
+        <v>363</v>
       </c>
       <c r="I195" s="136" t="n">
-        <v>3447</v>
+        <v>3570</v>
       </c>
       <c r="J195" s="137" t="n">
-        <v>1398.04</v>
+        <v>2458.12</v>
       </c>
       <c r="K195" s="137" t="n">
-        <v>1878</v>
-      </c>
-      <c r="L195" s="236">
+        <v>1814</v>
+      </c>
+      <c r="L195" s="235">
         <f>F195*(K195-J195)</f>
         <v/>
       </c>
@@ -15535,29 +15543,29 @@
       <c r="C196" s="138" t="n"/>
       <c r="D196" s="135" t="inlineStr">
         <is>
-          <t>穩懋(3105)</t>
+          <t>台燿(6274)</t>
         </is>
       </c>
       <c r="E196" s="136" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="F196" s="136" t="n">
-        <v>36</v>
+        <v>1</v>
       </c>
       <c r="G196" s="136" t="n">
-        <v>3365</v>
+        <v>3635</v>
       </c>
       <c r="H196" s="136" t="n">
-        <v>1713</v>
+        <v>188</v>
       </c>
       <c r="I196" s="136" t="n">
-        <v>1652</v>
+        <v>3447</v>
       </c>
       <c r="J196" s="137" t="n">
-        <v>467.4</v>
+        <v>1398.04</v>
       </c>
       <c r="K196" s="137" t="n">
-        <v>475.83</v>
+        <v>1878</v>
       </c>
       <c r="L196" s="236">
         <f>F196*(K196-J196)</f>
@@ -15570,29 +15578,29 @@
       <c r="C197" s="138" t="n"/>
       <c r="D197" s="135" t="inlineStr">
         <is>
-          <t>光寶科(2301)</t>
+          <t>穩懋(3105)</t>
         </is>
       </c>
       <c r="E197" s="136" t="n">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="F197" s="136" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="G197" s="136" t="n">
-        <v>2832</v>
+        <v>3365</v>
       </c>
       <c r="H197" s="136" t="n">
-        <v>918</v>
+        <v>1713</v>
       </c>
       <c r="I197" s="136" t="n">
-        <v>1914</v>
+        <v>1652</v>
       </c>
       <c r="J197" s="137" t="n">
-        <v>314.68</v>
+        <v>467.4</v>
       </c>
       <c r="K197" s="137" t="n">
-        <v>316.52</v>
+        <v>475.83</v>
       </c>
       <c r="L197" s="236">
         <f>F197*(K197-J197)</f>
@@ -15605,31 +15613,31 @@
       <c r="C198" s="138" t="n"/>
       <c r="D198" s="135" t="inlineStr">
         <is>
-          <t>欣興(3037)</t>
+          <t>光寶科(2301)</t>
         </is>
       </c>
       <c r="E198" s="136" t="n">
-        <v>26</v>
+        <v>90</v>
       </c>
       <c r="F198" s="136" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="G198" s="136" t="n">
-        <v>2550</v>
+        <v>2832</v>
       </c>
       <c r="H198" s="136" t="n">
-        <v>1919</v>
+        <v>918</v>
       </c>
       <c r="I198" s="136" t="n">
-        <v>631</v>
+        <v>1914</v>
       </c>
       <c r="J198" s="137" t="n">
-        <v>980.65</v>
+        <v>314.68</v>
       </c>
       <c r="K198" s="137" t="n">
-        <v>959.6</v>
-      </c>
-      <c r="L198" s="235">
+        <v>316.52</v>
+      </c>
+      <c r="L198" s="236">
         <f>F198*(K198-J198)</f>
         <v/>
       </c>
@@ -26093,7 +26101,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="207" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-09-02 17:25 | 9/9 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-09-02 18:14 | 9/9 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-09-03 03:13
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -2820,8 +2820,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G38" s="249" t="n">
-        <v>0.2035157242394799</v>
+      <c r="G38" s="244" t="n">
+        <v>0.2037160919806072</v>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
@@ -26101,7 +26101,7 @@
     <row r="484" ht="16.5" customHeight="1">
       <c r="A484" s="207" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-09-02 18:14 | 9/9 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-09-02 19:13 | 9/9 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-09-04 02:16
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -1655,7 +1655,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>💡 📌 一般共識 2408 / 6669 / 8046 (Q5 偏空, 中性信號)  |  避開 — 除權息 4 檔: 1203, 3661, 7780 ... | 明日恐處置 3 檔: 3625/4304/4971  |  訊號: 強偏空 (Q5 10%, hot=19)</t>
+          <t>💡 📌 一般共識 2408 / 6669 / 8046 (Q5 偏空, 中性信號)  |  避開 — 明日恐處置 3 檔: 3625/4304/4971  |  訊號: 強偏空 (Q5 10%, hot=19)</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2011,7 @@
         <v>13</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
@@ -2041,7 +2041,7 @@
         <v>10</v>
       </c>
       <c r="N20" s="17" t="n">
-        <v>39193</v>
+        <v>38483</v>
       </c>
     </row>
     <row r="21">
@@ -2525,7 +2525,7 @@
         </is>
       </c>
       <c r="G32" s="250" t="n">
-        <v>-199.54917</v>
+        <v>-199.32547</v>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
@@ -2543,7 +2543,7 @@
         </is>
       </c>
       <c r="G33" s="252" t="n">
-        <v>0.1706536496408914</v>
+        <v>0.170329424857283</v>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>23.6%</t>
+          <t>23.7%</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2654,11 +2654,11 @@
         </is>
       </c>
       <c r="D40" s="33" t="n">
-        <v>881453</v>
+        <v>870535</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>23.3%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>8.6%</t>
+          <t>8.7%</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>8.4%</t>
+          <t>8.5%</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="C53" s="40" t="inlineStr">
         <is>
-          <t>陳族元</t>
+          <t>迷你哥/松山哥</t>
         </is>
       </c>
       <c r="D53" s="40" t="inlineStr">
@@ -2959,12 +2959,12 @@
       </c>
       <c r="E53" s="40" t="inlineStr">
         <is>
-          <t>陳族元 今日買進 9 檔新標的 (過去從沒買過)</t>
+          <t>迷你哥/松山哥 今日買進 8 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F53" s="40" t="inlineStr">
         <is>
-          <t>9 檔</t>
+          <t>8 檔</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>迷你哥/松山哥</t>
+          <t>Tradow</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2986,12 +2986,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>迷你哥/松山哥 今日買進 8 檔新標的 (過去從沒買過)</t>
+          <t>Tradow 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>8 檔</t>
+          <t>6 檔</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="C55" s="40" t="inlineStr">
         <is>
-          <t>Tradow</t>
+          <t>布哥/n_nchang</t>
         </is>
       </c>
       <c r="D55" s="40" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="E55" s="40" t="inlineStr">
         <is>
-          <t>Tradow 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>布哥/n_nchang 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F55" s="40" t="inlineStr">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>布哥/n_nchang</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3040,7 +3040,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>布哥/n_nchang 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>竹科主力分點 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="C57" s="40" t="inlineStr">
         <is>
-          <t>竹科主力分點</t>
+          <t>陳律師</t>
         </is>
       </c>
       <c r="D57" s="40" t="inlineStr">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="E57" s="40" t="inlineStr">
         <is>
-          <t>竹科主力分點 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>陳律師 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F57" s="40" t="inlineStr">
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="C72" s="33" t="n">
-        <v>819686</v>
+        <v>809114</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3370,7 +3370,7 @@
         <v>40121</v>
       </c>
       <c r="J72" s="216" t="n">
-        <v>0.199874464124067</v>
+        <v>0.2024861026965552</v>
       </c>
     </row>
     <row r="73">
@@ -3820,7 +3820,7 @@
     <row r="86" ht="22" customHeight="1">
       <c r="B86" s="59" t="inlineStr">
         <is>
-          <t>▍ G. 注意股 (資料日 20260903)</t>
+          <t>▍ G. 注意股 (資料日 20260904)</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4210,7 @@
     <row r="108" ht="22" customHeight="1">
       <c r="B108" s="65" t="inlineStr">
         <is>
-          <t>▍ I. 未來 30 天除權息 (有效 77 檔, 已剔除過期)</t>
+          <t>▍ I. 未來 30 天除權息 (有效 74 檔, 已剔除過期)</t>
         </is>
       </c>
     </row>
@@ -4244,17 +4244,17 @@
     <row r="110">
       <c r="B110" t="inlineStr">
         <is>
-          <t>20260903</t>
+          <t>20260907</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>1203</t>
+          <t>00400A</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>味王</t>
+          <t>主動國泰動能高息</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -4263,23 +4263,23 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>1</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="111">
       <c r="B111" s="40" t="inlineStr">
         <is>
-          <t>20260903</t>
+          <t>20260907</t>
         </is>
       </c>
       <c r="C111" s="40" t="inlineStr">
         <is>
-          <t>3661</t>
+          <t>01010T</t>
         </is>
       </c>
       <c r="D111" s="40" t="inlineStr">
         <is>
-          <t>世芯-KY</t>
+          <t>京城樂富R1</t>
         </is>
       </c>
       <c r="E111" s="40" t="inlineStr">
@@ -4288,23 +4288,23 @@
         </is>
       </c>
       <c r="F111" s="40" t="n">
-        <v>32.551656</v>
+        <v>0.09872</v>
       </c>
     </row>
     <row r="112">
       <c r="B112" t="inlineStr">
         <is>
-          <t>20260903</t>
+          <t>20260907</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>7780</t>
+          <t>1466</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>大研生醫*</t>
+          <t>聚隆</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -4313,73 +4313,70 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>0.116588</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="113">
       <c r="B113" s="40" t="inlineStr">
         <is>
-          <t>20260903</t>
+          <t>20260907</t>
         </is>
       </c>
       <c r="C113" s="40" t="inlineStr">
         <is>
-          <t>8466</t>
+          <t>6533</t>
         </is>
       </c>
       <c r="D113" s="40" t="inlineStr">
         <is>
-          <t>美吉吉-KY</t>
+          <t>晶心科</t>
         </is>
       </c>
       <c r="E113" s="40" t="inlineStr">
         <is>
-          <t>息</t>
+          <t>權</t>
         </is>
       </c>
       <c r="F113" s="40" t="n">
-        <v>0.301938</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
-          <t>20260907</t>
+          <t>20260908</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>00400A</t>
+          <t>00940</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>主動國泰動能高息</t>
+          <t>元大台灣價值高息</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
           <t>息</t>
         </is>
-      </c>
-      <c r="F114" t="n">
-        <v>0.12</v>
       </c>
     </row>
     <row r="115">
       <c r="B115" s="40" t="inlineStr">
         <is>
-          <t>20260907</t>
+          <t>20260908</t>
         </is>
       </c>
       <c r="C115" s="40" t="inlineStr">
         <is>
-          <t>01010T</t>
+          <t>2379</t>
         </is>
       </c>
       <c r="D115" s="40" t="inlineStr">
         <is>
-          <t>京城樂富R1</t>
+          <t>瑞昱</t>
         </is>
       </c>
       <c r="E115" s="40" t="inlineStr">
@@ -4388,57 +4385,57 @@
         </is>
       </c>
       <c r="F115" s="40" t="n">
-        <v>0.09872</v>
+        <v>25</v>
       </c>
     </row>
     <row r="116">
       <c r="B116" t="inlineStr">
         <is>
-          <t>20260907</t>
+          <t>20260908</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>1466</t>
+          <t>2442</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>聚隆</t>
+          <t>新美齊</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>息</t>
+          <t>權息</t>
         </is>
       </c>
       <c r="F116" t="n">
-        <v>0.2</v>
+        <v>2.031861</v>
       </c>
     </row>
     <row r="117">
       <c r="B117" s="40" t="inlineStr">
         <is>
-          <t>20260907</t>
+          <t>20260908</t>
         </is>
       </c>
       <c r="C117" s="40" t="inlineStr">
         <is>
-          <t>6533</t>
+          <t>2706</t>
         </is>
       </c>
       <c r="D117" s="40" t="inlineStr">
         <is>
-          <t>晶心科</t>
+          <t>第一店</t>
         </is>
       </c>
       <c r="E117" s="40" t="inlineStr">
         <is>
-          <t>權</t>
+          <t>息</t>
         </is>
       </c>
       <c r="F117" s="40" t="n">
-        <v>0</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="118">
@@ -4449,18 +4446,21 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>00940</t>
+          <t>3312</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>元大台灣價值高息</t>
+          <t>弘憶股</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
           <t>息</t>
         </is>
+      </c>
+      <c r="F118" t="n">
+        <v>1.3</v>
       </c>
     </row>
     <row r="119">
@@ -4471,12 +4471,12 @@
       </c>
       <c r="C119" s="40" t="inlineStr">
         <is>
-          <t>2379</t>
+          <t>3622</t>
         </is>
       </c>
       <c r="D119" s="40" t="inlineStr">
         <is>
-          <t>瑞昱</t>
+          <t>洋華</t>
         </is>
       </c>
       <c r="E119" s="40" t="inlineStr">
@@ -4485,7 +4485,7 @@
         </is>
       </c>
       <c r="F119" s="40" t="n">
-        <v>25</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="120">
@@ -4496,12 +4496,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2442</t>
+          <t>8473</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>新美齊</t>
+          <t>山林水</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -4510,7 +4510,7 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>2.031861</v>
+        <v>0.782345</v>
       </c>
     </row>
     <row r="121">
@@ -4521,62 +4521,62 @@
       </c>
       <c r="C121" s="40" t="inlineStr">
         <is>
-          <t>2706</t>
+          <t>9933</t>
         </is>
       </c>
       <c r="D121" s="40" t="inlineStr">
         <is>
-          <t>第一店</t>
+          <t>中鼎</t>
         </is>
       </c>
       <c r="E121" s="40" t="inlineStr">
         <is>
-          <t>息</t>
+          <t>權息</t>
         </is>
       </c>
       <c r="F121" s="40" t="n">
-        <v>0.35</v>
+        <v>0.763056</v>
       </c>
     </row>
     <row r="122">
       <c r="B122" t="inlineStr">
         <is>
-          <t>20260908</t>
+          <t>20260909</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>3312</t>
+          <t>1438</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>弘憶股</t>
+          <t>三地開發</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>息</t>
+          <t>權息</t>
         </is>
       </c>
       <c r="F122" t="n">
-        <v>1.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="123">
       <c r="B123" s="40" t="inlineStr">
         <is>
-          <t>20260908</t>
+          <t>20260909</t>
         </is>
       </c>
       <c r="C123" s="40" t="inlineStr">
         <is>
-          <t>3622</t>
+          <t>3059</t>
         </is>
       </c>
       <c r="D123" s="40" t="inlineStr">
         <is>
-          <t>洋華</t>
+          <t>華晶科</t>
         </is>
       </c>
       <c r="E123" s="40" t="inlineStr">
@@ -4585,23 +4585,23 @@
         </is>
       </c>
       <c r="F123" s="40" t="n">
-        <v>3.2</v>
+        <v>0.998614</v>
       </c>
     </row>
     <row r="124">
       <c r="B124" t="inlineStr">
         <is>
-          <t>20260908</t>
+          <t>20260909</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>8473</t>
+          <t>3706</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>山林水</t>
+          <t>神達</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -4610,7 +4610,7 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>0.782345</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -4883,9 +4883,9 @@
       </c>
     </row>
     <row r="25">
-      <c r="C25" s="69" t="inlineStr">
-        <is>
-          <t>除權息 4 檔 (1203 / 3661 / 7780 ...)</t>
+      <c r="C25" s="71" t="inlineStr">
+        <is>
+          <t>今日無除權息</t>
         </is>
       </c>
     </row>
@@ -4906,7 +4906,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="C29" s="73" t="inlineStr">
         <is>
-          <t>-200 億 淨買</t>
+          <t>-199 億 淨買</t>
         </is>
       </c>
     </row>
@@ -7482,7 +7482,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="B3" s="99" t="inlineStr">
         <is>
-          <t>大牌分析師 近 25/25 交易日出手 1203 次 (345 檔), 風格分布: 隔日沖近似 34% / 當沖 14% / 留倉 52%, 漲停命中 3% (其中 🔒鎖漲停 2%), 前 5 大集中 18%, 長線部位 6% (4 檔), ⚠️ 處置股部位 12% (23 檔), 📦 連續囤貨 22 檔 (最長 12 天 00406A, 1 檔仍 active)。 主軸: 高頻交易/持續進場/📦 連續囤貨。</t>
+          <t>大牌分析師 近 25/25 交易日出手 1203 次 (345 檔), 風格分布: 隔日沖近似 34% / 當沖 14% / 留倉 52%, 漲停命中 3% (其中 🔒鎖漲停 2%), 前 5 大集中 18%, 長線部位 6% (4 檔), ⚠️ 處置股部位 9% (18 檔), 📦 連續囤貨 22 檔 (最長 12 天 00406A, 1 檔仍 active)。 主軸: 高頻交易/持續進場/📦 連續囤貨。</t>
         </is>
       </c>
     </row>
@@ -15060,7 +15060,7 @@
         </is>
       </c>
       <c r="E190" s="136" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F190" s="136" t="n">
         <v>4</v>
@@ -15075,7 +15075,7 @@
         <v>36163</v>
       </c>
       <c r="J190" s="137" t="n">
-        <v>1349.28</v>
+        <v>1344.34</v>
       </c>
       <c r="K190" s="137" t="n">
         <v>1342.5</v>
@@ -15095,10 +15095,10 @@
         </is>
       </c>
       <c r="E191" s="136" t="n">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="F191" s="136" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="G191" s="136" t="n">
         <v>6900</v>
@@ -15110,10 +15110,10 @@
         <v>5108</v>
       </c>
       <c r="J191" s="137" t="n">
-        <v>413.15</v>
+        <v>425.9</v>
       </c>
       <c r="K191" s="137" t="n">
-        <v>416.79</v>
+        <v>448.05</v>
       </c>
       <c r="L191" s="236">
         <f>F191*(K191-J191)</f>
@@ -15130,7 +15130,7 @@
         </is>
       </c>
       <c r="E192" s="136" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F192" s="136" t="n">
         <v>15</v>
@@ -15145,7 +15145,7 @@
         <v>5017</v>
       </c>
       <c r="J192" s="137" t="n">
-        <v>470.85</v>
+        <v>478.7</v>
       </c>
       <c r="K192" s="137" t="n">
         <v>484.53</v>
@@ -15200,10 +15200,10 @@
         </is>
       </c>
       <c r="E194" s="136" t="n">
-        <v>195</v>
+        <v>101</v>
       </c>
       <c r="F194" s="136" t="n">
-        <v>121</v>
+        <v>45</v>
       </c>
       <c r="G194" s="136" t="n">
         <v>4975</v>
@@ -15215,12 +15215,12 @@
         <v>2627</v>
       </c>
       <c r="J194" s="137" t="n">
-        <v>255.14</v>
+        <v>492.6</v>
       </c>
       <c r="K194" s="137" t="n">
-        <v>194.01</v>
-      </c>
-      <c r="L194" s="235">
+        <v>521.67</v>
+      </c>
+      <c r="L194" s="236">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -15235,10 +15235,10 @@
         </is>
       </c>
       <c r="E195" s="136" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F195" s="136" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G195" s="136" t="n">
         <v>4190</v>
@@ -15250,12 +15250,12 @@
         <v>3002</v>
       </c>
       <c r="J195" s="137" t="n">
-        <v>634.8200000000001</v>
+        <v>654.66</v>
       </c>
       <c r="K195" s="137" t="n">
-        <v>625</v>
-      </c>
-      <c r="L195" s="235">
+        <v>698.53</v>
+      </c>
+      <c r="L195" s="236">
         <f>F195*(K195-J195)</f>
         <v/>
       </c>
@@ -15270,10 +15270,10 @@
         </is>
       </c>
       <c r="E196" s="136" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F196" s="136" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G196" s="136" t="n">
         <v>3951</v>
@@ -15285,10 +15285,10 @@
         <v>2153</v>
       </c>
       <c r="J196" s="137" t="n">
-        <v>940.67</v>
+        <v>1067.78</v>
       </c>
       <c r="K196" s="137" t="n">
-        <v>899</v>
+        <v>1057.65</v>
       </c>
       <c r="L196" s="235">
         <f>F196*(K196-J196)</f>
@@ -15371,29 +15371,29 @@
       <c r="C199" s="138" t="n"/>
       <c r="D199" s="135" t="inlineStr">
         <is>
-          <t>晶豪科(3006)</t>
+          <t>富喬(1815)</t>
         </is>
       </c>
       <c r="E199" s="136" t="n">
-        <v>111</v>
+        <v>237</v>
       </c>
       <c r="F199" s="136" t="n">
-        <v>90</v>
+        <v>35</v>
       </c>
       <c r="G199" s="136" t="n">
-        <v>3075</v>
+        <v>2864</v>
       </c>
       <c r="H199" s="136" t="n">
-        <v>2493</v>
+        <v>441</v>
       </c>
       <c r="I199" s="136" t="n">
-        <v>582</v>
+        <v>2423</v>
       </c>
       <c r="J199" s="137" t="n">
-        <v>277</v>
+        <v>120.84</v>
       </c>
       <c r="K199" s="137" t="n">
-        <v>277</v>
+        <v>126</v>
       </c>
       <c r="L199" s="236">
         <f>F199*(K199-J199)</f>
@@ -25628,7 +25628,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="207" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-09-03 17:17 | 0/1 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-09-03 18:16 | 0/1 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-09-04 03:07
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -2011,7 +2011,7 @@
         <v>13</v>
       </c>
       <c r="F20" s="15" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
@@ -2041,7 +2041,7 @@
         <v>10</v>
       </c>
       <c r="N20" s="17" t="n">
-        <v>38483</v>
+        <v>39193</v>
       </c>
     </row>
     <row r="21">
@@ -2525,7 +2525,7 @@
         </is>
       </c>
       <c r="G32" s="250" t="n">
-        <v>-199.32547</v>
+        <v>-199.54917</v>
       </c>
     </row>
     <row r="33" ht="28" customHeight="1">
@@ -2543,7 +2543,7 @@
         </is>
       </c>
       <c r="G33" s="252" t="n">
-        <v>0.170329424857283</v>
+        <v>0.1706536496408914</v>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>23.7%</t>
+          <t>23.6%</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2654,11 +2654,11 @@
         </is>
       </c>
       <c r="D40" s="33" t="n">
-        <v>870535</v>
+        <v>881453</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>23.0%</t>
+          <t>23.3%</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>8.7%</t>
+          <t>8.6%</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>8.5%</t>
+          <t>8.4%</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="C53" s="40" t="inlineStr">
         <is>
-          <t>迷你哥/松山哥</t>
+          <t>陳族元</t>
         </is>
       </c>
       <c r="D53" s="40" t="inlineStr">
@@ -2959,12 +2959,12 @@
       </c>
       <c r="E53" s="40" t="inlineStr">
         <is>
-          <t>迷你哥/松山哥 今日買進 8 檔新標的 (過去從沒買過)</t>
+          <t>陳族元 今日買進 9 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F53" s="40" t="inlineStr">
         <is>
-          <t>8 檔</t>
+          <t>9 檔</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Tradow</t>
+          <t>迷你哥/松山哥</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2986,12 +2986,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Tradow 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>迷你哥/松山哥 今日買進 8 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>6 檔</t>
+          <t>8 檔</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="C55" s="40" t="inlineStr">
         <is>
-          <t>布哥/n_nchang</t>
+          <t>Tradow</t>
         </is>
       </c>
       <c r="D55" s="40" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="E55" s="40" t="inlineStr">
         <is>
-          <t>布哥/n_nchang 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>Tradow 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F55" s="40" t="inlineStr">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>竹科主力分點</t>
+          <t>布哥/n_nchang</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3040,7 +3040,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>竹科主力分點 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>布哥/n_nchang 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="C57" s="40" t="inlineStr">
         <is>
-          <t>陳律師</t>
+          <t>竹科主力分點</t>
         </is>
       </c>
       <c r="D57" s="40" t="inlineStr">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="E57" s="40" t="inlineStr">
         <is>
-          <t>陳律師 今日買進 6 檔新標的 (過去從沒買過)</t>
+          <t>竹科主力分點 今日買進 6 檔新標的 (過去從沒買過)</t>
         </is>
       </c>
       <c r="F57" s="40" t="inlineStr">
@@ -3343,7 +3343,7 @@
         </is>
       </c>
       <c r="C72" s="33" t="n">
-        <v>809114</v>
+        <v>819686</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3370,7 +3370,7 @@
         <v>40121</v>
       </c>
       <c r="J72" s="216" t="n">
-        <v>0.2024861026965552</v>
+        <v>0.199874464124067</v>
       </c>
     </row>
     <row r="73">
@@ -4906,7 +4906,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="C29" s="73" t="inlineStr">
         <is>
-          <t>-199 億 淨買</t>
+          <t>-200 億 淨買</t>
         </is>
       </c>
     </row>
@@ -15060,7 +15060,7 @@
         </is>
       </c>
       <c r="E190" s="136" t="n">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F190" s="136" t="n">
         <v>4</v>
@@ -15075,7 +15075,7 @@
         <v>36163</v>
       </c>
       <c r="J190" s="137" t="n">
-        <v>1344.34</v>
+        <v>1349.28</v>
       </c>
       <c r="K190" s="137" t="n">
         <v>1342.5</v>
@@ -15095,10 +15095,10 @@
         </is>
       </c>
       <c r="E191" s="136" t="n">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="F191" s="136" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G191" s="136" t="n">
         <v>6900</v>
@@ -15110,10 +15110,10 @@
         <v>5108</v>
       </c>
       <c r="J191" s="137" t="n">
-        <v>425.9</v>
+        <v>413.15</v>
       </c>
       <c r="K191" s="137" t="n">
-        <v>448.05</v>
+        <v>416.79</v>
       </c>
       <c r="L191" s="236">
         <f>F191*(K191-J191)</f>
@@ -15130,7 +15130,7 @@
         </is>
       </c>
       <c r="E192" s="136" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F192" s="136" t="n">
         <v>15</v>
@@ -15145,7 +15145,7 @@
         <v>5017</v>
       </c>
       <c r="J192" s="137" t="n">
-        <v>478.7</v>
+        <v>470.85</v>
       </c>
       <c r="K192" s="137" t="n">
         <v>484.53</v>
@@ -15200,10 +15200,10 @@
         </is>
       </c>
       <c r="E194" s="136" t="n">
-        <v>101</v>
+        <v>195</v>
       </c>
       <c r="F194" s="136" t="n">
-        <v>45</v>
+        <v>121</v>
       </c>
       <c r="G194" s="136" t="n">
         <v>4975</v>
@@ -15215,12 +15215,12 @@
         <v>2627</v>
       </c>
       <c r="J194" s="137" t="n">
-        <v>492.6</v>
+        <v>255.14</v>
       </c>
       <c r="K194" s="137" t="n">
-        <v>521.67</v>
-      </c>
-      <c r="L194" s="236">
+        <v>194.01</v>
+      </c>
+      <c r="L194" s="235">
         <f>F194*(K194-J194)</f>
         <v/>
       </c>
@@ -15235,10 +15235,10 @@
         </is>
       </c>
       <c r="E195" s="136" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F195" s="136" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G195" s="136" t="n">
         <v>4190</v>
@@ -15250,12 +15250,12 @@
         <v>3002</v>
       </c>
       <c r="J195" s="137" t="n">
-        <v>654.66</v>
+        <v>634.8200000000001</v>
       </c>
       <c r="K195" s="137" t="n">
-        <v>698.53</v>
-      </c>
-      <c r="L195" s="236">
+        <v>625</v>
+      </c>
+      <c r="L195" s="235">
         <f>F195*(K195-J195)</f>
         <v/>
       </c>
@@ -15270,10 +15270,10 @@
         </is>
       </c>
       <c r="E196" s="136" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="F196" s="136" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G196" s="136" t="n">
         <v>3951</v>
@@ -15285,10 +15285,10 @@
         <v>2153</v>
       </c>
       <c r="J196" s="137" t="n">
-        <v>1067.78</v>
+        <v>940.67</v>
       </c>
       <c r="K196" s="137" t="n">
-        <v>1057.65</v>
+        <v>899</v>
       </c>
       <c r="L196" s="235">
         <f>F196*(K196-J196)</f>
@@ -15371,29 +15371,29 @@
       <c r="C199" s="138" t="n"/>
       <c r="D199" s="135" t="inlineStr">
         <is>
-          <t>富喬(1815)</t>
+          <t>晶豪科(3006)</t>
         </is>
       </c>
       <c r="E199" s="136" t="n">
-        <v>237</v>
+        <v>111</v>
       </c>
       <c r="F199" s="136" t="n">
-        <v>35</v>
+        <v>90</v>
       </c>
       <c r="G199" s="136" t="n">
-        <v>2864</v>
+        <v>3075</v>
       </c>
       <c r="H199" s="136" t="n">
-        <v>441</v>
+        <v>2493</v>
       </c>
       <c r="I199" s="136" t="n">
-        <v>2423</v>
+        <v>582</v>
       </c>
       <c r="J199" s="137" t="n">
-        <v>120.84</v>
+        <v>277</v>
       </c>
       <c r="K199" s="137" t="n">
-        <v>126</v>
+        <v>277</v>
       </c>
       <c r="L199" s="236">
         <f>F199*(K199-J199)</f>
@@ -25628,7 +25628,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="207" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-09-03 18:16 | 0/1 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-09-03 19:07 | 0/1 success</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔒 [FULL] Daily chip data 2026-09-05 02:49
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-09.xlsx
+++ b/data/reports/chip_radar_2026-09.xlsx
@@ -24,7 +24,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="29">
+  <numFmts count="30">
     <numFmt numFmtId="164" formatCode="0%&quot; (13/13 ・昨100/5d100)&quot;"/>
     <numFmt numFmtId="165" formatCode="+0&quot; 億 (昨-177/5d-99)&quot;;-0&quot; 億 (昨-177/5d-99)&quot;;0&quot; 億&quot;"/>
     <numFmt numFmtId="166" formatCode="0&quot; 檔 +63億 &quot;&quot;(昨15/5d11)&quot;"/>
@@ -54,6 +54,7 @@
     <numFmt numFmtId="190" formatCode="0&quot; 檔 +34億 &quot;&quot;(昨14/5d13)&quot;"/>
     <numFmt numFmtId="191" formatCode="0.0%&quot; 市-446億 &quot;&quot;(昨17/5d18)&quot;"/>
     <numFmt numFmtId="192" formatCode="0&quot; 檔 +36億 &quot;&quot;(昨14/5d13)&quot;"/>
+    <numFmt numFmtId="193" formatCode="0.0%&quot; 市-444億 &quot;&quot;(昨17/5d18)&quot;"/>
   </numFmts>
   <fonts count="54">
     <font>
@@ -642,7 +643,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="260">
+  <cellXfs count="261">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1249,6 +1250,9 @@
     <xf numFmtId="192" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="193" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2557,8 +2561,8 @@
           <t>Q4 追蹤佔比</t>
         </is>
       </c>
-      <c r="G32" s="258" t="n">
-        <v>0.1700160365736953</v>
+      <c r="G32" s="260" t="n">
+        <v>0.1701493816780536</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
@@ -3835,7 +3839,7 @@
     <row r="85" ht="22" customHeight="1">
       <c r="B85" s="59" t="inlineStr">
         <is>
-          <t>▍ G. 注意股 (資料日 20260904)</t>
+          <t>▍ G. 注意股 (資料日 20260905)</t>
         </is>
       </c>
     </row>
@@ -4376,6 +4380,9 @@
         <is>
           <t>息</t>
         </is>
+      </c>
+      <c r="F113" t="n">
+        <v>0.055</v>
       </c>
     </row>
     <row r="114">
@@ -7533,7 +7540,7 @@
     <row r="3" ht="28" customHeight="1">
       <c r="B3" s="99" t="inlineStr">
         <is>
-          <t>大牌分析師 近 26/26 交易日出手 1255 次 (353 檔), 風格分布: 隔日沖近似 34% / 當沖 14% / 留倉 52%, 漲停命中 3% (其中 🔒鎖漲停 2%), 前 5 大集中 18%, 長線部位 6% (5 檔), ⚠️ 處置股部位 9% (19 檔), 📦 連續囤貨 23 檔 (最長 12 天 00406A, 3 檔仍 active)。 主軸: 分散布局/高頻交易/持續進場/📦 連續囤貨。</t>
+          <t>大牌分析師 近 26/26 交易日出手 1255 次 (353 檔), 風格分布: 隔日沖近似 34% / 當沖 14% / 留倉 52%, 漲停命中 3% (其中 🔒鎖漲停 2%), 前 5 大集中 18%, 長線部位 6% (5 檔), ⚠️ 處置股部位 10% (19 檔), 📦 連續囤貨 23 檔 (最長 12 天 00406A, 3 檔仍 active)。 主軸: 分散布局/高頻交易/持續進場/📦 連續囤貨。</t>
         </is>
       </c>
     </row>
@@ -26074,7 +26081,7 @@
     <row r="485" ht="16.5" customHeight="1">
       <c r="A485" s="207" t="inlineStr">
         <is>
-          <t>ⓘ histock top-buyer 資料 fetched @ 2026-09-04 17:59 | 0/17 success</t>
+          <t>ⓘ histock top-buyer 資料 fetched @ 2026-09-04 18:49 | 0/17 success</t>
         </is>
       </c>
     </row>

</xml_diff>